<commit_message>
model: charity seed and local investor rows in the funding stack
Claude-Session: https://claude.ai/code/session_01R3VSDVSHrTTdt9iVs9Smn8
</commit_message>
<xml_diff>
--- a/docs/venue-model-andover-unit-28.xlsx
+++ b/docs/venue-model-andover-unit-28.xlsx
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -4135,23 +4135,23 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="C14" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="D14" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="E14" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="F14" s="26">
-        <f>-Capital!$B$40</f>
+        <f>-Capital!$B$43</f>
         <v/>
       </c>
       <c r="G14" s="28">
@@ -4250,7 +4250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -4624,15 +4624,15 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Founders, community investors, Crowdfunder</t>
+          <t>Local sports charity: seed for Phase 1 and match funding</t>
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>150000</v>
+        <v>25000</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Crowdfunder + Sport England match up to £15k; CIC ltd by shares for investors</t>
+          <t>Known to Adam; pays the survey, pre-app and engineer so no director funds Phase 1 personally</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4644,15 +4644,15 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Donations, naming-rights advance</t>
+          <t>Local private investors introduced by the charity (patient capital)</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>100000</v>
+        <v>250000</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Year-0 sponsorship paid up front</t>
+          <t>Capped-dividend shares in a CIC ltd by shares, a rent-deposit guarantee, or donations via the charitable arm. If it comes as a 6% loan instead, add about £34k a year of service</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4664,124 +4664,164 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LTA padel loan (Quick Access / Facility Loan)</t>
+          <t>Crowdfunder with Sport England match</t>
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>200000</v>
+        <v>30000</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>£25k–£250k at 5%, up to 10 years</t>
+          <t>Match up to £15k; also a demand test</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>loan</t>
+          <t>grant/equity</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Donations, naming-rights advance</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Year-0 sponsorship paid up front</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>grant/equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LTA padel loan (Quick Access / Facility Loan)</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>£25k–£250k at 5%, up to 10 years</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>loan</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Charity Bank / Triodos / Pitch Together loan</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B31" s="11" t="n">
         <v>400000</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Pitch Together £25k–£300k at 6%; Charity Bank larger</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>loan</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Total grants, donations and equity</t>
-        </is>
-      </c>
-      <c r="B31" s="26">
-        <f>SUMIF(D19:D29,"grant/equity",B19:B29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Total loans</t>
-        </is>
-      </c>
-      <c r="B32" s="26">
-        <f>SUMIF(D19:D29,"loan",B19:B29)</f>
-        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Total sources</t>
-        </is>
-      </c>
-      <c r="B33" s="29">
-        <f>B31+B32</f>
+          <t>Total grants, donations and equity</t>
+        </is>
+      </c>
+      <c r="B33" s="26">
+        <f>SUMIF(D19:D31,"grant/equity",B19:B31)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>Total loans</t>
+        </is>
+      </c>
+      <c r="B34" s="26">
+        <f>SUMIF(D19:D31,"loan",B19:B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Total sources</t>
+        </is>
+      </c>
+      <c r="B35" s="29">
+        <f>B33+B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>Surplus / (gap)</t>
         </is>
       </c>
-      <c r="B34" s="29">
-        <f>B33-B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="B36" s="29">
+        <f>B35-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Grants and donations as % of capital</t>
         </is>
       </c>
-      <c r="B36" s="30">
-        <f>B31/B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="B38" s="30">
+        <f>B33/B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Loan service</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Loan principal</t>
         </is>
       </c>
-      <c r="B39" s="26">
-        <f>B32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="B42" s="26">
+        <f>B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Annual repayment (annuity)</t>
         </is>
       </c>
-      <c r="B40" s="12">
-        <f>IF(B39=0,0,-PMT(Inputs!$E$126,Inputs!$E$127,B39))</f>
+      <c r="B43" s="12">
+        <f>IF(B42=0,0,-PMT(Inputs!$E$126,Inputs!$E$127,B42))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Momentum Ltd sheet on teams x fee x 10-week seasons; Basingstoke growth route
Claude-Session: https://claude.ai/code/session_01R3VSDVSHrTTdt9iVs9Smn8
</commit_message>
<xml_diff>
--- a/docs/venue-model-andover-unit-28.xlsx
+++ b/docs/venue-model-andover-unit-28.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,7 +122,10 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4836,7 +4839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -4855,7 +4858,7 @@
     <row r="2">
       <c r="A2" s="25" t="inlineStr">
         <is>
-          <t>Today, school halls cost Momentum about £24 per court-hour. The CIC must charge an arm's-length rate, so Momentum's league margin changes. This sheet shows what has to move.</t>
+          <t>School halls cost Momentum about £24 per court-hour. The CIC must charge an arm's-length rate. At £450 a season the league absorbs that easily; the venue's value to Momentum is room to grow past 24 teams in Andover, alongside new town leagues.</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4867,7 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Today (Xero FY26)</t>
+          <t>Today (24 teams, £450, Xero FY26)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -4874,249 +4877,264 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>In the CIC, new fees</t>
+          <t>In the CIC, 36 teams at £480</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Evening court-hours per week</t>
+          <t>Teams in the Andover women's league</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" s="7">
-        <f>Inputs!$E$17</f>
-        <v/>
-      </c>
-      <c r="D6" s="7">
-        <f>Inputs!$E$17</f>
-        <v/>
+        <v>24</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Weeks per year</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C7" s="7">
-        <f>Inputs!$E$31</f>
-        <v/>
-      </c>
-      <c r="D7" s="7">
-        <f>Inputs!$E$31</f>
-        <v/>
+          <t>Fee per team per season</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>450</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>450</v>
+      </c>
+      <c r="D7" s="31" t="n">
+        <v>480</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rate per court-hour paid</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>24</v>
-      </c>
-      <c r="C8" s="13">
-        <f>Inputs!$E$19*(1-Inputs!$E$30)</f>
-        <v/>
-      </c>
-      <c r="D8" s="13">
-        <f>Inputs!$E$19*(1-Inputs!$E$30)</f>
-        <v/>
+          <t>Seasons per year (each about 10 weeks)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Matches per court-hour</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>1.5</v>
+          <t>Matches per week (teams / 2)</t>
+        </is>
+      </c>
+      <c r="B9" s="32">
+        <f>B6/2</f>
+        <v/>
+      </c>
+      <c r="C9" s="32">
+        <f>C6/2</f>
+        <v/>
+      </c>
+      <c r="D9" s="32">
+        <f>D6/2</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fee per team per match</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <v>25</v>
+          <t>Matches per court-hour</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Other direct costs per match (umpires, insurance, prizes)</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="C11" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <v>6</v>
+          <t>Court-hours per week (matches / matches per court-hour)</t>
+        </is>
+      </c>
+      <c r="B11" s="32">
+        <f>B9/B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="32">
+        <f>C9/C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="32">
+        <f>D9/D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Weeks per year (seasons x 10)</t>
+        </is>
+      </c>
+      <c r="B12" s="33">
+        <f>B8*10</f>
+        <v/>
+      </c>
+      <c r="C12" s="33">
+        <f>C8*10</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>D8*10</f>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Matches per year</t>
-        </is>
-      </c>
-      <c r="B13" s="31">
-        <f>B6*B7*B9</f>
-        <v/>
-      </c>
-      <c r="C13" s="31">
-        <f>C6*C7*C9</f>
-        <v/>
-      </c>
-      <c r="D13" s="31">
-        <f>D6*D7*D9</f>
+          <t>Rate per court-hour paid</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="C13" s="34">
+        <f>Inputs!$E$19*(1-Inputs!$E$30)</f>
+        <v/>
+      </c>
+      <c r="D13" s="34">
+        <f>Inputs!$E$19*(1-Inputs!$E$30)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>League income (2 teams per match)</t>
-        </is>
-      </c>
-      <c r="B14" s="26">
-        <f>B13*2*B10</f>
-        <v/>
-      </c>
-      <c r="C14" s="26">
-        <f>C13*2*C10</f>
-        <v/>
-      </c>
-      <c r="D14" s="26">
-        <f>D13*2*D10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Court hire paid</t>
-        </is>
-      </c>
-      <c r="B15" s="26">
-        <f>-B6*B7*B8</f>
-        <v/>
-      </c>
-      <c r="C15" s="26">
-        <f>-C6*C7*C8</f>
-        <v/>
-      </c>
-      <c r="D15" s="26">
-        <f>-D6*D7*D8</f>
-        <v/>
+          <t>Other direct costs per match (umpires, insurance, prizes)</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Other direct costs</t>
+          <t>League income (teams x fee x seasons)</t>
         </is>
       </c>
       <c r="B16" s="26">
-        <f>-B13*B11</f>
+        <f>B6*B7*B8</f>
         <v/>
       </c>
       <c r="C16" s="26">
-        <f>-C13*C11</f>
+        <f>C6*C7*C8</f>
         <v/>
       </c>
       <c r="D16" s="26">
-        <f>-D13*D11</f>
+        <f>D6*D7*D8</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>League gross profit</t>
-        </is>
-      </c>
-      <c r="B17" s="12">
-        <f>SUM(B14:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="12">
-        <f>SUM(C14:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="12">
-        <f>SUM(D14:D16)</f>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Court hire</t>
+        </is>
+      </c>
+      <c r="B17" s="26">
+        <f>-B11*B12*B13</f>
+        <v/>
+      </c>
+      <c r="C17" s="26">
+        <f>-C11*C12*C13</f>
+        <v/>
+      </c>
+      <c r="D17" s="26">
+        <f>-D11*D12*D13</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gross margin</t>
-        </is>
-      </c>
-      <c r="B18" s="30">
-        <f>IF(B14=0,0,B17/B14)</f>
-        <v/>
-      </c>
-      <c r="C18" s="30">
-        <f>IF(C14=0,0,C17/C14)</f>
-        <v/>
-      </c>
-      <c r="D18" s="30">
-        <f>IF(D14=0,0,D17/D14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>Reference points: Xero FY26 league sales £43,781 and venue hire £14,647. Commercial leagues (Play Netball, Go Mammoth) charge £8–10 per player per match, about £56–70 per team. Momentum's £18 per team per match is the cheapest in the market by a distance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
+          <t>Other direct costs</t>
+        </is>
+      </c>
+      <c r="B18" s="26">
+        <f>-B9*B12*B14</f>
+        <v/>
+      </c>
+      <c r="C18" s="26">
+        <f>-C9*C12*C14</f>
+        <v/>
+      </c>
+      <c r="D18" s="26">
+        <f>-D9*D12*D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>League gross profit</t>
+        </is>
+      </c>
+      <c r="B19" s="12">
+        <f>SUM(B16:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="12">
+        <f>SUM(C16:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="12">
+        <f>SUM(D16:D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>Reference points: 24 teams x £450 x 4 ten-week seasons = £43,200 against Xero FY26 league sales of £43,781, i.e. £45 per team per match. Total venue hire £14,647 covers the league (about 8 court-hours a week) plus mixed, training, Netball Hour and pay-to-play. Commercial leagues charge £56–70 per team per match. Growth routes: more Andover divisions in the hub, and more towns (Basingstoke next) on the same model with the hub as home for finals, tournaments and training.</t>
+        </is>
+      </c>
+    </row>
     <row r="22"/>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+    <row r="23"/>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Governance: directors common to Momentum Ltd and the CIC must declare the conflict, the CIC board needs independent members, and the court-hire contract must be at the published rate. Funders and the CIC Regulator look for exactly this.</t>
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26"/>
+    <row r="27"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:D3"/>
-    <mergeCell ref="A20:D22"/>
-    <mergeCell ref="A24:D26"/>
+    <mergeCell ref="A25:D27"/>
+    <mergeCell ref="A21:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5440,7 +5458,7 @@
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Momentum Netball Ltd can stay independent and block-book courts from the CIC (mode 2 on Inputs). The Momentum Ltd sheet shows the effect on its league margin: at an arm's-length rate its £18 per team per match no longer covers the court, so fees rise or the league grows.</t>
+          <t>Momentum Netball Ltd can stay independent and block-book courts from the CIC (mode 2 on Inputs). The Momentum Ltd sheet shows the league at 24 teams x £450 x 4 ten-week seasons: the arm's-length court rate costs it about £5.4k a year; growth to 36 teams more than covers it.</t>
         </is>
       </c>
     </row>

</xml_diff>